<commit_message>
Remove test-account passwords from test-case workbooks, ignore backups
Passwords are now read only from the local .env; the workbooks reference it.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/test-cases/Aros_Regression_Admin.xlsx
+++ b/docs/test-cases/Aros_Regression_Admin.xlsx
@@ -154,7 +154,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -176,11 +176,55 @@
         <color rgb="00BDBDBD"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00BDBDBD"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00BDBDBD"/>
+      </right>
+      <top style="thin">
+        <color rgb="00BDBDBD"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00BDBDBD"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00BDBDBD"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00BDBDBD"/>
+      </right>
+      <top style="thin">
+        <color rgb="00BDBDBD"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00BDBDBD"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="36">
+  <cellXfs count="38">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -255,6 +299,8 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -806,6 +852,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -838,7 +885,7 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>Логин: +998998987882   Пароль: Sh2004Sh</t>
+          <t>Логин: +998998987882   Пароль: &lt;пароль в .env&gt; в .env&gt;</t>
         </is>
       </c>
     </row>
@@ -873,12 +920,12 @@
         </is>
       </c>
       <c r="B9" s="5" t="inlineStr"/>
-      <c r="C9" s="6" t="n"/>
-      <c r="D9" s="6" t="n"/>
-      <c r="E9" s="6" t="n"/>
-      <c r="F9" s="6" t="n"/>
-      <c r="G9" s="6" t="n"/>
-      <c r="H9" s="6" t="n"/>
+      <c r="C9" s="36" t="n"/>
+      <c r="D9" s="36" t="n"/>
+      <c r="E9" s="36" t="n"/>
+      <c r="F9" s="36" t="n"/>
+      <c r="G9" s="36" t="n"/>
+      <c r="H9" s="37" t="n"/>
       <c r="J9" s="7" t="inlineStr">
         <is>
           <t>← жёлтые поля заполняются перед каждым прогоном</t>
@@ -892,12 +939,12 @@
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr"/>
-      <c r="C10" s="6" t="n"/>
-      <c r="D10" s="6" t="n"/>
-      <c r="E10" s="6" t="n"/>
-      <c r="F10" s="6" t="n"/>
-      <c r="G10" s="6" t="n"/>
-      <c r="H10" s="6" t="n"/>
+      <c r="C10" s="36" t="n"/>
+      <c r="D10" s="36" t="n"/>
+      <c r="E10" s="36" t="n"/>
+      <c r="F10" s="36" t="n"/>
+      <c r="G10" s="36" t="n"/>
+      <c r="H10" s="37" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
@@ -906,12 +953,12 @@
         </is>
       </c>
       <c r="B11" s="5" t="inlineStr"/>
-      <c r="C11" s="6" t="n"/>
-      <c r="D11" s="6" t="n"/>
-      <c r="E11" s="6" t="n"/>
-      <c r="F11" s="6" t="n"/>
-      <c r="G11" s="6" t="n"/>
-      <c r="H11" s="6" t="n"/>
+      <c r="C11" s="36" t="n"/>
+      <c r="D11" s="36" t="n"/>
+      <c r="E11" s="36" t="n"/>
+      <c r="F11" s="36" t="n"/>
+      <c r="G11" s="36" t="n"/>
+      <c r="H11" s="37" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="8" t="inlineStr">
@@ -2635,6 +2682,7 @@
         <v/>
       </c>
     </row>
+    <row r="40"/>
     <row r="41">
       <c r="A41" s="8" t="inlineStr">
         <is>
@@ -2958,7 +3006,7 @@
       </c>
       <c r="I2" s="27" t="inlineStr">
         <is>
-          <t>+998998987882 / Sh2004Sh</t>
+          <t>+998998987882 / &lt;пароль в .env&gt;</t>
         </is>
       </c>
       <c r="J2" s="27" t="inlineStr">
@@ -14727,6 +14775,7 @@
         </is>
       </c>
     </row>
+    <row r="7"/>
     <row r="8">
       <c r="B8" s="34" t="inlineStr">
         <is>

</xml_diff>